<commit_message>
Add Istanbul official price research to v0.6
</commit_message>
<xml_diff>
--- a/GPT전달내용/travel_cost_research_pilot_v0.6_2026-10-03.xlsx
+++ b/GPT전달내용/travel_cost_research_pilot_v0.6_2026-10-03.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="조사 기준" sheetId="1" r:id="R3fca274aa310402c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="도시 우선순위" sheetId="2" r:id="R7800e90a0e0f4284"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="가격 표본" sheetId="3" r:id="Rcf74d50c62ff42b8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="음식 추천" sheetId="4" r:id="R0209576022b649fb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="도시 초안" sheetId="5" r:id="Ra94712776ed44c09"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="다음 조사 큐" sheetId="6" r:id="R1ec33ba484834dd8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="조사 기준" sheetId="1" r:id="Rbc3cfa38dc164fa9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="도시 우선순위" sheetId="2" r:id="R36dc0a9813dc4fed"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="가격 표본" sheetId="3" r:id="Rf6759dbdcfac4e79"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="음식 추천" sheetId="4" r:id="Rf199e2286b814dc6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="도시 초안" sheetId="5" r:id="R5baa29bfad5f4e3a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="다음 조사 큐" sheetId="6" r:id="Reeefc44559314157"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -334,8 +334,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="PriceObservationTable" displayName="PriceObservationTable" ref="A4:U190" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A4:U190"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="PriceObservationTable" displayName="PriceObservationTable" ref="A4:U222" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A4:U222"/>
   <x:tableColumns count="21">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="국가"/>
@@ -364,8 +364,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="FoodRecommendationTable" displayName="FoodRecommendationTable" ref="A4:K44" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A4:K44"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="FoodRecommendationTable" displayName="FoodRecommendationTable" ref="A4:K49" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A4:K49"/>
   <x:tableColumns count="11">
     <x:tableColumn id="1" name="국가"/>
     <x:tableColumn id="2" name="도시"/>
@@ -1764,7 +1764,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R336edce5c82f4564"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc55b13e7ab734d01"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -13968,6 +13968,2086 @@
         <x:v>공식몰 상품 목록에 갓 책갈피 10,000원.</x:v>
       </x:c>
     </x:row>
+    <x:row r="191" ht="36" customHeight="1">
+      <x:c r="A191" t="str">
+        <x:v>IST-TR-001</x:v>
+      </x:c>
+      <x:c r="B191" t="str">
+        <x:v>튀르키예</x:v>
+      </x:c>
+      <x:c r="C191" t="str">
+        <x:v>이스탄불</x:v>
+      </x:c>
+      <x:c r="D191" t="str">
+        <x:v>교통</x:v>
+      </x:c>
+      <x:c r="E191" t="str">
+        <x:v>도시철도 1회권</x:v>
+      </x:c>
+      <x:c r="F191" t="str">
+        <x:v>Metro İstanbul 익명 İstanbulkart 일반 편도</x:v>
+      </x:c>
+      <x:c r="G191" t="str">
+        <x:v>Metro Istanbul Anonymous Istanbulkart Full Fare</x:v>
+      </x:c>
+      <x:c r="H191" s="55" t="n">
+        <x:v>46.2</x:v>
+      </x:c>
+      <x:c r="I191" s="55" t="n">
+        <x:v>46.2</x:v>
+      </x:c>
+      <x:c r="J191" t="str">
+        <x:v>TRY</x:v>
+      </x:c>
+      <x:c r="K191" t="str">
+        <x:v>1회</x:v>
+      </x:c>
+      <x:c r="L191" t="str">
+        <x:v>고정형</x:v>
+      </x:c>
+      <x:c r="M191" t="str">
+        <x:v>성인</x:v>
+      </x:c>
+      <x:c r="N191" t="str">
+        <x:v>A 공식</x:v>
+      </x:c>
+      <x:c r="O191" t="str">
+        <x:v>예</x:v>
+      </x:c>
+      <x:c r="P191" t="str">
+        <x:v>확정 1차</x:v>
+      </x:c>
+      <x:c r="Q191" s="51" t="n">
+        <x:v>46298</x:v>
+      </x:c>
+      <x:c r="R191" t="str">
+        <x:v>2026-10-03 확인</x:v>
+      </x:c>
+      <x:c r="S191" t="str">
+        <x:v>Metro İstanbul</x:v>
+      </x:c>
+      <x:c r="T191" t="str">
+        <x:v>https://www.metro.istanbul/seferdurumlari/biletucretleri</x:v>
+      </x:c>
+      <x:c r="U191" s="23" t="str">
+        <x:v>운영사 공식 요금표의 익명 카드 일반 운임 46.20 TRY.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="192" ht="36" customHeight="1">
+      <x:c r="A192" t="str">
+        <x:v>IST-TR-002</x:v>
+      </x:c>
+      <x:c r="B192" t="str">
+        <x:v>튀르키예</x:v>
+      </x:c>
+      <x:c r="C192" t="str">
+        <x:v>이스탄불</x:v>
+      </x:c>
+      <x:c r="D192" t="str">
+        <x:v>교통</x:v>
+      </x:c>
+      <x:c r="E192" t="str">
+        <x:v>도시철도 1회권</x:v>
+      </x:c>
+      <x:c r="F192" t="str">
+        <x:v>Metro İstanbul 1회권 전자티켓</x:v>
+      </x:c>
+      <x:c r="G192" t="str">
+        <x:v>Metro Istanbul One-Pass Electronic Ticket</x:v>
+      </x:c>
+      <x:c r="H192" s="55" t="n">
+        <x:v>65</x:v>
+      </x:c>
+      <x:c r="I192" s="55" t="n">
+        <x:v>65</x:v>
+      </x:c>
+      <x:c r="J192" t="str">
+        <x:v>TRY</x:v>
+      </x:c>
+      <x:c r="K192" t="str">
+        <x:v>1회</x:v>
+      </x:c>
+      <x:c r="L192" t="str">
+        <x:v>고정형</x:v>
+      </x:c>
+      <x:c r="M192" t="str">
+        <x:v>일반</x:v>
+      </x:c>
+      <x:c r="N192" t="str">
+        <x:v>A 공식</x:v>
+      </x:c>
+      <x:c r="O192" t="str">
+        <x:v>예</x:v>
+      </x:c>
+      <x:c r="P192" t="str">
+        <x:v>확정 1차</x:v>
+      </x:c>
+      <x:c r="Q192" s="51" t="n">
+        <x:v>46298</x:v>
+      </x:c>
+      <x:c r="R192" t="str">
+        <x:v>2026-10-03 확인</x:v>
+      </x:c>
+      <x:c r="S192" t="str">
+        <x:v>Metro İstanbul</x:v>
+      </x:c>
+      <x:c r="T192" t="str">
+        <x:v>https://www.metro.istanbul/seferdurumlari/biletucretleri</x:v>
+      </x:c>
+      <x:c r="U192" s="23" t="str">
+        <x:v>운영사 공식 요금표의 Bir Geçişlik Kart 65 TRY.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="193" ht="36" customHeight="1">
+      <x:c r="A193" t="str">
+        <x:v>IST-TR-003</x:v>
+      </x:c>
+      <x:c r="B193" t="str">
+        <x:v>튀르키예</x:v>
+      </x:c>
+      <x:c r="C193" t="str">
+        <x:v>이스탄불</x:v>
+      </x:c>
+      <x:c r="D193" t="str">
+        <x:v>교통</x:v>
+      </x:c>
+      <x:c r="E193" t="str">
+        <x:v>페리 1회권</x:v>
+      </x:c>
+      <x:c r="F193" t="str">
+        <x:v>Şehir Hatları 카라쿄이–카드쾨이 편도</x:v>
+      </x:c>
+      <x:c r="G193" t="str">
+        <x:v>Şehir Hatları Karaköy–Kadıköy One Way</x:v>
+      </x:c>
+      <x:c r="H193" s="55" t="n">
+        <x:v>65.21</x:v>
+      </x:c>
+      <x:c r="I193" s="55" t="n">
+        <x:v>65.21</x:v>
+      </x:c>
+      <x:c r="J193" t="str">
+        <x:v>TRY</x:v>
+      </x:c>
+      <x:c r="K193" t="str">
+        <x:v>1회</x:v>
+      </x:c>
+      <x:c r="L193" t="str">
+        <x:v>고정형</x:v>
+      </x:c>
+      <x:c r="M193" t="str">
+        <x:v>성인</x:v>
+      </x:c>
+      <x:c r="N193" t="str">
+        <x:v>A 공식</x:v>
+      </x:c>
+      <x:c r="O193" t="str">
+        <x:v>예</x:v>
+      </x:c>
+      <x:c r="P193" t="str">
+        <x:v>확정 1차</x:v>
+      </x:c>
+      <x:c r="Q193" s="51" t="n">
+        <x:v>46298</x:v>
+      </x:c>
+      <x:c r="R193" t="str">
+        <x:v>2026-10-03 확인</x:v>
+      </x:c>
+      <x:c r="S193" t="str">
+        <x:v>Şehir Hatları</x:v>
+      </x:c>
+      <x:c r="T193" t="str">
+        <x:v>https://sehirhatlari.istanbul/tr/ucret-tarifeleri/vapur-hatlari-79</x:v>
+      </x:c>
+      <x:c r="U193" s="23" t="str">
+        <x:v>공식 중심 노선표에서 Karaköy–Kadıköy 일반(İstanbulkart Tam) 65.21 TRY.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="194" ht="36" customHeight="1">
+      <x:c r="A194" t="str">
+        <x:v>IST-AP-001</x:v>
+      </x:c>
+      <x:c r="B194" t="str">
+        <x:v>튀르키예</x:v>
+      </x:c>
+      <x:c r="C194" t="str">
+        <x:v>이스탄불</x:v>
+      </x:c>
+      <x:c r="D194" t="str">
+        <x:v>공항이동</x:v>
+      </x:c>
+      <x:c r="E194" t="str">
+        <x:v>공항버스</x:v>
+      </x:c>
+      <x:c r="F194" t="str">
+        <x:v>HAVAİST 술탄아흐메트–이스탄불 공항 편도</x:v>
+      </x:c>
+      <x:c r="G194" t="str">
+        <x:v>HAVAİST Sultanahmet–Istanbul Airport One Way</x:v>
+      </x:c>
+      <x:c r="H194" s="55" t="n">
+        <x:v>470</x:v>
+      </x:c>
+      <x:c r="I194" s="55" t="n">
+        <x:v>470</x:v>
+      </x:c>
+      <x:c r="J194" t="str">
+        <x:v>TRY</x:v>
+      </x:c>
+      <x:c r="K194" t="str">
+        <x:v>성인 1인 편도</x:v>
+      </x:c>
+      <x:c r="L194" t="str">
+        <x:v>고정형</x:v>
+      </x:c>
+      <x:c r="M194" t="str">
+        <x:v>일반</x:v>
+      </x:c>
+      <x:c r="N194" t="str">
+        <x:v>A 공식</x:v>
+      </x:c>
+      <x:c r="O194" t="str">
+        <x:v>예</x:v>
+      </x:c>
+      <x:c r="P194" t="str">
+        <x:v>확정 1차</x:v>
+      </x:c>
+      <x:c r="Q194" s="51" t="n">
+        <x:v>46298</x:v>
+      </x:c>
+      <x:c r="R194" t="str">
+        <x:v>2026-05-17 게시</x:v>
+      </x:c>
+      <x:c r="S194" t="str">
+        <x:v>HAVAİST</x:v>
+      </x:c>
+      <x:c r="T194" t="str">
+        <x:v>https://blog.hava.ist/havaist-sultanahmet-hatti-yeniden-hizmette/</x:v>
+      </x:c>
+      <x:c r="U194" s="23" t="str">
+        <x:v>공식 운영자 공지의 Sultanahmet–IST 노선 편도 승차권 470 TRY.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="195" ht="36" customHeight="1">
+      <x:c r="A195" t="str">
+        <x:v>IST-AP-002</x:v>
+      </x:c>
+      <x:c r="B195" t="str">
+        <x:v>튀르키예</x:v>
+      </x:c>
+      <x:c r="C195" t="str">
+        <x:v>이스탄불</x:v>
+      </x:c>
+      <x:c r="D195" t="str">
+        <x:v>공항이동</x:v>
+      </x:c>
+      <x:c r="E195" t="str">
+        <x:v>공항버스</x:v>
+      </x:c>
+      <x:c r="F195" t="str">
+        <x:v>HAVAİST 술탄가지/오토가르–이스탄불 공항 편도</x:v>
+      </x:c>
+      <x:c r="G195" t="str">
+        <x:v>HAVAİST Sultangazi/Otogar–Istanbul Airport One Way</x:v>
+      </x:c>
+      <x:c r="H195" s="55" t="n">
+        <x:v>370</x:v>
+      </x:c>
+      <x:c r="I195" s="55" t="n">
+        <x:v>370</x:v>
+      </x:c>
+      <x:c r="J195" t="str">
+        <x:v>TRY</x:v>
+      </x:c>
+      <x:c r="K195" t="str">
+        <x:v>성인 1인 편도</x:v>
+      </x:c>
+      <x:c r="L195" t="str">
+        <x:v>고정형</x:v>
+      </x:c>
+      <x:c r="M195" t="str">
+        <x:v>일반</x:v>
+      </x:c>
+      <x:c r="N195" t="str">
+        <x:v>A 공식</x:v>
+      </x:c>
+      <x:c r="O195" t="str">
+        <x:v>예</x:v>
+      </x:c>
+      <x:c r="P195" t="str">
+        <x:v>확정 1차</x:v>
+      </x:c>
+      <x:c r="Q195" s="51" t="n">
+        <x:v>46298</x:v>
+      </x:c>
+      <x:c r="R195" t="str">
+        <x:v>2026-09-08 게시</x:v>
+      </x:c>
+      <x:c r="S195" t="str">
+        <x:v>HAVAİST</x:v>
+      </x:c>
+      <x:c r="T195" t="str">
+        <x:v>https://blog.hava.ist/sultangazi-istanbul-havalimani-havaist/</x:v>
+      </x:c>
+      <x:c r="U195" s="23" t="str">
+        <x:v>공식 운영자 공지의 Otogar–IST 노선에서 술탄가지 정차지 이용 시 편도 370 TRY.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="196" ht="36" customHeight="1">
+      <x:c r="A196" t="str">
+        <x:v>IST-FD-001</x:v>
+      </x:c>
+      <x:c r="B196" t="str">
+        <x:v>튀르키예</x:v>
+      </x:c>
+      <x:c r="C196" t="str">
+        <x:v>이스탄불</x:v>
+      </x:c>
+      <x:c r="D196" t="str">
+        <x:v>외식</x:v>
+      </x:c>
+      <x:c r="E196" t="str">
+        <x:v>메뉴 표본</x:v>
+      </x:c>
+      <x:c r="F196" t="str">
+        <x:v>Konak Restaurant 닭갈비구이 Tavuk Pirzola</x:v>
+      </x:c>
+      <x:c r="G196" t="str">
+        <x:v>Konak Restaurant Grilled Chicken Chops</x:v>
+      </x:c>
+      <x:c r="H196" s="55" t="n">
+        <x:v>460</x:v>
+      </x:c>
+      <x:c r="I196" s="55" t="n">
+        <x:v>460</x:v>
+      </x:c>
+      <x:c r="J196" t="str">
+        <x:v>TRY</x:v>
+      </x:c>
+      <x:c r="K196" t="str">
+        <x:v>1인분</x:v>
+      </x:c>
+      <x:c r="L196" t="str">
+        <x:v>메뉴형</x:v>
+      </x:c>
+      <x:c r="M196" t="str">
+        <x:v>일반</x:v>
+      </x:c>
+      <x:c r="N196" t="str">
+        <x:v>A 공식</x:v>
+      </x:c>
+      <x:c r="O196" t="str">
+        <x:v>예</x:v>
+      </x:c>
+      <x:c r="P196" t="str">
+        <x:v>확정 1차</x:v>
+      </x:c>
+      <x:c r="Q196" s="51" t="n">
+        <x:v>46298</x:v>
+      </x:c>
+      <x:c r="R196" t="str">
+        <x:v>2026-10-03 확인</x:v>
+      </x:c>
+      <x:c r="S196" t="str">
+        <x:v>Konak Restaurant</x:v>
+      </x:c>
+      <x:c r="T196" t="str">
+        <x:v>https://www.konakrestaurant.com/menu.html</x:v>
+      </x:c>
+      <x:c r="U196" s="23" t="str">
+        <x:v>공식 메뉴의 Tavuk Pirzola 항목가 460 TRY. Büyükada 소재.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="197" ht="36" customHeight="1">
+      <x:c r="A197" t="str">
+        <x:v>IST-FD-002</x:v>
+      </x:c>
+      <x:c r="B197" t="str">
+        <x:v>튀르키예</x:v>
+      </x:c>
+      <x:c r="C197" t="str">
+        <x:v>이스탄불</x:v>
+      </x:c>
+      <x:c r="D197" t="str">
+        <x:v>외식</x:v>
+      </x:c>
+      <x:c r="E197" t="str">
+        <x:v>메뉴 표본</x:v>
+      </x:c>
+      <x:c r="F197" t="str">
+        <x:v>Saklı Kubbe 차으 케밥 2꼬치 100g</x:v>
+      </x:c>
+      <x:c r="G197" t="str">
+        <x:v>Saklı Kubbe Cağ Kebab, 2 Skewers, 100 g</x:v>
+      </x:c>
+      <x:c r="H197" s="55" t="n">
+        <x:v>580</x:v>
+      </x:c>
+      <x:c r="I197" s="55" t="n">
+        <x:v>580</x:v>
+      </x:c>
+      <x:c r="J197" t="str">
+        <x:v>TRY</x:v>
+      </x:c>
+      <x:c r="K197" t="str">
+        <x:v>1인분 100g</x:v>
+      </x:c>
+      <x:c r="L197" t="str">
+        <x:v>메뉴형</x:v>
+      </x:c>
+      <x:c r="M197" t="str">
+        <x:v>일반</x:v>
+      </x:c>
+      <x:c r="N197" t="str">
+        <x:v>A 공식</x:v>
+      </x:c>
+      <x:c r="O197" t="str">
+        <x:v>예</x:v>
+      </x:c>
+      <x:c r="P197" t="str">
+        <x:v>확정 1차</x:v>
+      </x:c>
+      <x:c r="Q197" s="51" t="n">
+        <x:v>46298</x:v>
+      </x:c>
+      <x:c r="R197" t="str">
+        <x:v>2026-05-12 적용</x:v>
+      </x:c>
+      <x:c r="S197" t="str">
+        <x:v>Saklı Kubbe</x:v>
+      </x:c>
+      <x:c r="T197" t="str">
+        <x:v>https://www.saklikubbe.com/menu/</x:v>
+      </x:c>
+      <x:c r="U197" s="23" t="str">
+        <x:v>공식 메뉴에 2꼬치 100g 580 TRY, 가격 변경일 2026-05-12.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="198" ht="36" customHeight="1">
+      <x:c r="A198" t="str">
+        <x:v>IST-FD-003</x:v>
+      </x:c>
+      <x:c r="B198" t="str">
+        <x:v>튀르키예</x:v>
+      </x:c>
+      <x:c r="C198" t="str">
+        <x:v>이스탄불</x:v>
+      </x:c>
+      <x:c r="D198" t="str">
+        <x:v>외식</x:v>
+      </x:c>
+      <x:c r="E198" t="str">
+        <x:v>메뉴 표본</x:v>
+      </x:c>
+      <x:c r="F198" t="str">
+        <x:v>Pino Gare Tavuk Şiş</x:v>
+      </x:c>
+      <x:c r="G198" t="str">
+        <x:v>Pino Gare Chicken Shish</x:v>
+      </x:c>
+      <x:c r="H198" s="55" t="n">
+        <x:v>975</x:v>
+      </x:c>
+      <x:c r="I198" s="55" t="n">
+        <x:v>975</x:v>
+      </x:c>
+      <x:c r="J198" t="str">
+        <x:v>TRY</x:v>
+      </x:c>
+      <x:c r="K198" t="str">
+        <x:v>1인분</x:v>
+      </x:c>
+      <x:c r="L198" t="str">
+        <x:v>메뉴형</x:v>
+      </x:c>
+      <x:c r="M198" t="str">
+        <x:v>일반</x:v>
+      </x:c>
+      <x:c r="N198" t="str">
+        <x:v>A 공식</x:v>
+      </x:c>
+      <x:c r="O198" t="str">
+        <x:v>예</x:v>
+      </x:c>
+      <x:c r="P198" t="str">
+        <x:v>확정 1차</x:v>
+      </x:c>
+      <x:c r="Q198" s="51" t="n">
+        <x:v>46298</x:v>
+      </x:c>
+      <x:c r="R198" t="str">
+        <x:v>2026-10-03 확인</x:v>
+      </x:c>
+      <x:c r="S198" t="str">
+        <x:v>Pino Gare Rooftop Restaurant</x:v>
+      </x:c>
+      <x:c r="T198" t="str">
+        <x:v>https://pinogareroofrestaurant.com/tr/menu</x:v>
+      </x:c>
+      <x:c r="U198" s="23" t="str">
+        <x:v>공식 메뉴의 tavuk but şiş 세트 975 TRY.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="199" ht="36" customHeight="1">
+      <x:c r="A199" t="str">
+        <x:v>IST-FD-004</x:v>
+      </x:c>
+      <x:c r="B199" t="str">
+        <x:v>튀르키예</x:v>
+      </x:c>
+      <x:c r="C199" t="str">
+        <x:v>이스탄불</x:v>
+      </x:c>
+      <x:c r="D199" t="str">
+        <x:v>외식</x:v>
+      </x:c>
+      <x:c r="E199" t="str">
+        <x:v>메뉴 표본</x:v>
+      </x:c>
+      <x:c r="F199" t="str">
+        <x:v>Lokanta Lobi Lobi Köftesi</x:v>
+      </x:c>
+      <x:c r="G199" t="str">
+        <x:v>Lokanta Lobi Lobi Meatballs</x:v>
+      </x:c>
+      <x:c r="H199" s="55" t="n">
+        <x:v>1400</x:v>
+      </x:c>
+      <x:c r="I199" s="55" t="n">
+        <x:v>1400</x:v>
+      </x:c>
+      <x:c r="J199" t="str">
+        <x:v>TRY</x:v>
+      </x:c>
+      <x:c r="K199" t="str">
+        <x:v>1인분</x:v>
+      </x:c>
+      <x:c r="L199" t="str">
+        <x:v>메뉴형</x:v>
+      </x:c>
+      <x:c r="M199" t="str">
+        <x:v>일반</x:v>
+      </x:c>
+      <x:c r="N199" t="str">
+        <x:v>A 공식</x:v>
+      </x:c>
+      <x:c r="O199" t="str">
+        <x:v>예</x:v>
+      </x:c>
+      <x:c r="P199" t="str">
+        <x:v>확정 1차</x:v>
+      </x:c>
+      <x:c r="Q199" s="51" t="n">
+        <x:v>46298</x:v>
+      </x:c>
+      <x:c r="R199" t="str">
+        <x:v>2026-10-03 확인</x:v>
+      </x:c>
+      <x:c r="S199" t="str">
+        <x:v>Lokanta Lobi</x:v>
+      </x:c>
+      <x:c r="T199" t="str">
+        <x:v>https://lokantalobi.com/menu/</x:v>
+      </x:c>
+      <x:c r="U199" s="23" t="str">
+        <x:v>공식 메뉴의 구운 소고기 köfte와 감자 메뉴 1,400 TRY.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="200" ht="36" customHeight="1">
+      <x:c r="A200" t="str">
+        <x:v>IST-FD-005</x:v>
+      </x:c>
+      <x:c r="B200" t="str">
+        <x:v>튀르키예</x:v>
+      </x:c>
+      <x:c r="C200" t="str">
+        <x:v>이스탄불</x:v>
+      </x:c>
+      <x:c r="D200" t="str">
+        <x:v>외식</x:v>
+      </x:c>
+      <x:c r="E200" t="str">
+        <x:v>메뉴 표본</x:v>
+      </x:c>
+      <x:c r="F200" t="str">
+        <x:v>Cafe Şamdan Adana Kebap 150g</x:v>
+      </x:c>
+      <x:c r="G200" t="str">
+        <x:v>Cafe Şamdan Adana Kebab, 150 g</x:v>
+      </x:c>
+      <x:c r="H200" s="55" t="n">
+        <x:v>450</x:v>
+      </x:c>
+      <x:c r="I200" s="55" t="n">
+        <x:v>450</x:v>
+      </x:c>
+      <x:c r="J200" t="str">
+        <x:v>TRY</x:v>
+      </x:c>
+      <x:c r="K200" t="str">
+        <x:v>1인분 150g</x:v>
+      </x:c>
+      <x:c r="L200" t="str">
+        <x:v>메뉴형</x:v>
+      </x:c>
+      <x:c r="M200" t="str">
+        <x:v>일반</x:v>
+      </x:c>
+      <x:c r="N200" t="str">
+        <x:v>A 공식</x:v>
+      </x:c>
+      <x:c r="O200" t="str">
+        <x:v>예</x:v>
+      </x:c>
+      <x:c r="P200" t="str">
+        <x:v>확정 1차</x:v>
+      </x:c>
+      <x:c r="Q200" s="51" t="n">
+        <x:v>46298</x:v>
+      </x:c>
+      <x:c r="R200" t="str">
+        <x:v>2026-04-11 적용</x:v>
+      </x:c>
+      <x:c r="S200" t="str">
+        <x:v>Cafe Şamdan</x:v>
+      </x:c>
+      <x:c r="T200" t="str">
+        <x:v>https://www.cafesamdan.com.tr/</x:v>
+      </x:c>
+      <x:c r="U200" s="23" t="str">
+        <x:v>공식 QR 메뉴의 Adana kebap 150g, 450 TRY. 가격 변경일 2026-04-11.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="201" ht="36" customHeight="1">
+      <x:c r="A201" t="str">
+        <x:v>IST-SN-001</x:v>
+      </x:c>
+      <x:c r="B201" t="str">
+        <x:v>튀르키예</x:v>
+      </x:c>
+      <x:c r="C201" t="str">
+        <x:v>이스탄불</x:v>
+      </x:c>
+      <x:c r="D201" t="str">
+        <x:v>외식</x:v>
+      </x:c>
+      <x:c r="E201" t="str">
+        <x:v>음료</x:v>
+      </x:c>
+      <x:c r="F201" t="str">
+        <x:v>Saklı Kubbe Beyoğlu Gazozu</x:v>
+      </x:c>
+      <x:c r="G201" t="str">
+        <x:v>Saklı Kubbe Beyoğlu Gazoz</x:v>
+      </x:c>
+      <x:c r="H201" s="55" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="I201" s="55" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="J201" t="str">
+        <x:v>TRY</x:v>
+      </x:c>
+      <x:c r="K201" t="str">
+        <x:v>1병 250ml</x:v>
+      </x:c>
+      <x:c r="L201" t="str">
+        <x:v>메뉴형</x:v>
+      </x:c>
+      <x:c r="M201" t="str">
+        <x:v>일반</x:v>
+      </x:c>
+      <x:c r="N201" t="str">
+        <x:v>A 공식</x:v>
+      </x:c>
+      <x:c r="O201" t="str">
+        <x:v>예</x:v>
+      </x:c>
+      <x:c r="P201" t="str">
+        <x:v>확정 1차</x:v>
+      </x:c>
+      <x:c r="Q201" s="51" t="n">
+        <x:v>46298</x:v>
+      </x:c>
+      <x:c r="R201" t="str">
+        <x:v>2026-05-12 적용</x:v>
+      </x:c>
+      <x:c r="S201" t="str">
+        <x:v>Saklı Kubbe</x:v>
+      </x:c>
+      <x:c r="T201" t="str">
+        <x:v>https://www.saklikubbe.com/menu/</x:v>
+      </x:c>
+      <x:c r="U201" s="23" t="str">
+        <x:v>공식 메뉴의 Beyoğlu Gazozu 250ml 100 TRY.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="202" ht="36" customHeight="1">
+      <x:c r="A202" t="str">
+        <x:v>IST-SN-002</x:v>
+      </x:c>
+      <x:c r="B202" t="str">
+        <x:v>튀르키예</x:v>
+      </x:c>
+      <x:c r="C202" t="str">
+        <x:v>이스탄불</x:v>
+      </x:c>
+      <x:c r="D202" t="str">
+        <x:v>외식</x:v>
+      </x:c>
+      <x:c r="E202" t="str">
+        <x:v>음료</x:v>
+      </x:c>
+      <x:c r="F202" t="str">
+        <x:v>Saklı Kubbe Eker Tombul Ayran</x:v>
+      </x:c>
+      <x:c r="G202" t="str">
+        <x:v>Saklı Kubbe Eker Tombul Ayran</x:v>
+      </x:c>
+      <x:c r="H202" s="55" t="n">
+        <x:v>80</x:v>
+      </x:c>
+      <x:c r="I202" s="55" t="n">
+        <x:v>80</x:v>
+      </x:c>
+      <x:c r="J202" t="str">
+        <x:v>TRY</x:v>
+      </x:c>
+      <x:c r="K202" t="str">
+        <x:v>1병 293ml</x:v>
+      </x:c>
+      <x:c r="L202" t="str">
+        <x:v>메뉴형</x:v>
+      </x:c>
+      <x:c r="M202" t="str">
+        <x:v>일반</x:v>
+      </x:c>
+      <x:c r="N202" t="str">
+        <x:v>A 공식</x:v>
+      </x:c>
+      <x:c r="O202" t="str">
+        <x:v>예</x:v>
+      </x:c>
+      <x:c r="P202" t="str">
+        <x:v>확정 1차</x:v>
+      </x:c>
+      <x:c r="Q202" s="51" t="n">
+        <x:v>46298</x:v>
+      </x:c>
+      <x:c r="R202" t="str">
+        <x:v>2026-05-12 적용</x:v>
+      </x:c>
+      <x:c r="S202" t="str">
+        <x:v>Saklı Kubbe</x:v>
+      </x:c>
+      <x:c r="T202" t="str">
+        <x:v>https://www.saklikubbe.com/menu/</x:v>
+      </x:c>
+      <x:c r="U202" s="23" t="str">
+        <x:v>공식 메뉴의 Eker Tombul Ayran 293ml 80 TRY.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="203" ht="36" customHeight="1">
+      <x:c r="A203" t="str">
+        <x:v>IST-SN-003</x:v>
+      </x:c>
+      <x:c r="B203" t="str">
+        <x:v>튀르키예</x:v>
+      </x:c>
+      <x:c r="C203" t="str">
+        <x:v>이스탄불</x:v>
+      </x:c>
+      <x:c r="D203" t="str">
+        <x:v>외식</x:v>
+      </x:c>
+      <x:c r="E203" t="str">
+        <x:v>음료</x:v>
+      </x:c>
+      <x:c r="F203" t="str">
+        <x:v>Saklı Kubbe 데운 차 한 잔</x:v>
+      </x:c>
+      <x:c r="G203" t="str">
+        <x:v>Saklı Kubbe Brewed Tea, Glass</x:v>
+      </x:c>
+      <x:c r="H203" s="55" t="n">
+        <x:v>35</x:v>
+      </x:c>
+      <x:c r="I203" s="55" t="n">
+        <x:v>35</x:v>
+      </x:c>
+      <x:c r="J203" t="str">
+        <x:v>TRY</x:v>
+      </x:c>
+      <x:c r="K203" t="str">
+        <x:v>1잔</x:v>
+      </x:c>
+      <x:c r="L203" t="str">
+        <x:v>메뉴형</x:v>
+      </x:c>
+      <x:c r="M203" t="str">
+        <x:v>일반</x:v>
+      </x:c>
+      <x:c r="N203" t="str">
+        <x:v>A 공식</x:v>
+      </x:c>
+      <x:c r="O203" t="str">
+        <x:v>예</x:v>
+      </x:c>
+      <x:c r="P203" t="str">
+        <x:v>확정 1차</x:v>
+      </x:c>
+      <x:c r="Q203" s="51" t="n">
+        <x:v>46298</x:v>
+      </x:c>
+      <x:c r="R203" t="str">
+        <x:v>2026-05-12 적용</x:v>
+      </x:c>
+      <x:c r="S203" t="str">
+        <x:v>Saklı Kubbe</x:v>
+      </x:c>
+      <x:c r="T203" t="str">
+        <x:v>https://www.saklikubbe.com/menu/</x:v>
+      </x:c>
+      <x:c r="U203" s="23" t="str">
+        <x:v>공식 메뉴의 Demleme Bardak Çayı 35 TRY.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="204" ht="36" customHeight="1">
+      <x:c r="A204" t="str">
+        <x:v>IST-AL-001</x:v>
+      </x:c>
+      <x:c r="B204" t="str">
+        <x:v>튀르키예</x:v>
+      </x:c>
+      <x:c r="C204" t="str">
+        <x:v>이스탄불</x:v>
+      </x:c>
+      <x:c r="D204" t="str">
+        <x:v>외식</x:v>
+      </x:c>
+      <x:c r="E204" t="str">
+        <x:v>주류</x:v>
+      </x:c>
+      <x:c r="F204" t="str">
+        <x:v>Lokanta Lobi Mercan 라키</x:v>
+      </x:c>
+      <x:c r="G204" t="str">
+        <x:v>Lokanta Lobi Mercan Rakı</x:v>
+      </x:c>
+      <x:c r="H204" s="55" t="n">
+        <x:v>550</x:v>
+      </x:c>
+      <x:c r="I204" s="55" t="n">
+        <x:v>550</x:v>
+      </x:c>
+      <x:c r="J204" t="str">
+        <x:v>TRY</x:v>
+      </x:c>
+      <x:c r="K204" t="str">
+        <x:v>1잔 6cl</x:v>
+      </x:c>
+      <x:c r="L204" t="str">
+        <x:v>메뉴형</x:v>
+      </x:c>
+      <x:c r="M204" t="str">
+        <x:v>성인</x:v>
+      </x:c>
+      <x:c r="N204" t="str">
+        <x:v>A 공식</x:v>
+      </x:c>
+      <x:c r="O204" t="str">
+        <x:v>예</x:v>
+      </x:c>
+      <x:c r="P204" t="str">
+        <x:v>확정 1차</x:v>
+      </x:c>
+      <x:c r="Q204" s="51" t="n">
+        <x:v>46298</x:v>
+      </x:c>
+      <x:c r="R204" t="str">
+        <x:v>2026-10-03 확인</x:v>
+      </x:c>
+      <x:c r="S204" t="str">
+        <x:v>Lokanta Lobi</x:v>
+      </x:c>
+      <x:c r="T204" t="str">
+        <x:v>https://lokantalobi.com/menu/</x:v>
+      </x:c>
+      <x:c r="U204" s="23" t="str">
+        <x:v>공식 메뉴의 Rakı bölümünde bardak 6cl Mercan 550 TRY.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="205" ht="36" customHeight="1">
+      <x:c r="A205" t="str">
+        <x:v>IST-AL-002</x:v>
+      </x:c>
+      <x:c r="B205" t="str">
+        <x:v>튀르키예</x:v>
+      </x:c>
+      <x:c r="C205" t="str">
+        <x:v>이스탄불</x:v>
+      </x:c>
+      <x:c r="D205" t="str">
+        <x:v>외식</x:v>
+      </x:c>
+      <x:c r="E205" t="str">
+        <x:v>주류</x:v>
+      </x:c>
+      <x:c r="F205" t="str">
+        <x:v>Lokanta Lobi Efes 생맥주</x:v>
+      </x:c>
+      <x:c r="G205" t="str">
+        <x:v>Lokanta Lobi Efes Draft Beer</x:v>
+      </x:c>
+      <x:c r="H205" s="55" t="n">
+        <x:v>300</x:v>
+      </x:c>
+      <x:c r="I205" s="55" t="n">
+        <x:v>300</x:v>
+      </x:c>
+      <x:c r="J205" t="str">
+        <x:v>TRY</x:v>
+      </x:c>
+      <x:c r="K205" t="str">
+        <x:v>1잔 33cl</x:v>
+      </x:c>
+      <x:c r="L205" t="str">
+        <x:v>메뉴형</x:v>
+      </x:c>
+      <x:c r="M205" t="str">
+        <x:v>성인</x:v>
+      </x:c>
+      <x:c r="N205" t="str">
+        <x:v>A 공식</x:v>
+      </x:c>
+      <x:c r="O205" t="str">
+        <x:v>예</x:v>
+      </x:c>
+      <x:c r="P205" t="str">
+        <x:v>확정 1차</x:v>
+      </x:c>
+      <x:c r="Q205" s="51" t="n">
+        <x:v>46298</x:v>
+      </x:c>
+      <x:c r="R205" t="str">
+        <x:v>2026-10-03 확인</x:v>
+      </x:c>
+      <x:c r="S205" t="str">
+        <x:v>Lokanta Lobi</x:v>
+      </x:c>
+      <x:c r="T205" t="str">
+        <x:v>https://lokantalobi.com/menu/</x:v>
+      </x:c>
+      <x:c r="U205" s="23" t="str">
+        <x:v>공식 메뉴의 fıçı Efes 33cl 300 TRY.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="206" ht="36" customHeight="1">
+      <x:c r="A206" t="str">
+        <x:v>IST-AL-003</x:v>
+      </x:c>
+      <x:c r="B206" t="str">
+        <x:v>튀르키예</x:v>
+      </x:c>
+      <x:c r="C206" t="str">
+        <x:v>이스탄불</x:v>
+      </x:c>
+      <x:c r="D206" t="str">
+        <x:v>외식</x:v>
+      </x:c>
+      <x:c r="E206" t="str">
+        <x:v>주류</x:v>
+      </x:c>
+      <x:c r="F206" t="str">
+        <x:v>Lokanta Lobi Efes 무글루텐 맥주</x:v>
+      </x:c>
+      <x:c r="G206" t="str">
+        <x:v>Lokanta Lobi Efes Gluten-Free Beer</x:v>
+      </x:c>
+      <x:c r="H206" s="55" t="n">
+        <x:v>450</x:v>
+      </x:c>
+      <x:c r="I206" s="55" t="n">
+        <x:v>450</x:v>
+      </x:c>
+      <x:c r="J206" t="str">
+        <x:v>TRY</x:v>
+      </x:c>
+      <x:c r="K206" t="str">
+        <x:v>1병 50cl</x:v>
+      </x:c>
+      <x:c r="L206" t="str">
+        <x:v>메뉴형</x:v>
+      </x:c>
+      <x:c r="M206" t="str">
+        <x:v>성인</x:v>
+      </x:c>
+      <x:c r="N206" t="str">
+        <x:v>A 공식</x:v>
+      </x:c>
+      <x:c r="O206" t="str">
+        <x:v>예</x:v>
+      </x:c>
+      <x:c r="P206" t="str">
+        <x:v>확정 1차</x:v>
+      </x:c>
+      <x:c r="Q206" s="51" t="n">
+        <x:v>46298</x:v>
+      </x:c>
+      <x:c r="R206" t="str">
+        <x:v>2026-10-03 확인</x:v>
+      </x:c>
+      <x:c r="S206" t="str">
+        <x:v>Lokanta Lobi</x:v>
+      </x:c>
+      <x:c r="T206" t="str">
+        <x:v>https://lokantalobi.com/menu/</x:v>
+      </x:c>
+      <x:c r="U206" s="23" t="str">
+        <x:v>공식 메뉴의 Efes Glutensiz 50cl 450 TRY.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="207" ht="36" customHeight="1">
+      <x:c r="A207" t="str">
+        <x:v>IST-SV-001</x:v>
+      </x:c>
+      <x:c r="B207" t="str">
+        <x:v>튀르키예</x:v>
+      </x:c>
+      <x:c r="C207" t="str">
+        <x:v>이스탄불</x:v>
+      </x:c>
+      <x:c r="D207" t="str">
+        <x:v>기념품</x:v>
+      </x:c>
+      <x:c r="E207" t="str">
+        <x:v>식품</x:v>
+      </x:c>
+      <x:c r="F207" t="str">
+        <x:v>Karaköy Güllüoğlu Galata Akşamı 바클라바 500g</x:v>
+      </x:c>
+      <x:c r="G207" t="str">
+        <x:v>Karaköy Güllüoğlu Galata Akşamı Baklava, 500 g</x:v>
+      </x:c>
+      <x:c r="H207" s="55" t="n">
+        <x:v>1170</x:v>
+      </x:c>
+      <x:c r="I207" s="55" t="n">
+        <x:v>1170</x:v>
+      </x:c>
+      <x:c r="J207" t="str">
+        <x:v>TRY</x:v>
+      </x:c>
+      <x:c r="K207" t="str">
+        <x:v>1상자 500g</x:v>
+      </x:c>
+      <x:c r="L207" t="str">
+        <x:v>고정형</x:v>
+      </x:c>
+      <x:c r="M207" t="str">
+        <x:v>일반</x:v>
+      </x:c>
+      <x:c r="N207" t="str">
+        <x:v>A 공식</x:v>
+      </x:c>
+      <x:c r="O207" t="str">
+        <x:v>예</x:v>
+      </x:c>
+      <x:c r="P207" t="str">
+        <x:v>확정 1차</x:v>
+      </x:c>
+      <x:c r="Q207" s="51" t="n">
+        <x:v>46298</x:v>
+      </x:c>
+      <x:c r="R207" t="str">
+        <x:v>2026-10-03 확인</x:v>
+      </x:c>
+      <x:c r="S207" t="str">
+        <x:v>Karaköy Güllüoğlu</x:v>
+      </x:c>
+      <x:c r="T207" t="str">
+        <x:v>https://www.karakoygulluoglu.com/kent-miras%C4%B1-kutular-galata-ak%C5%9Fam%C4%B1-500-gr.-baklava</x:v>
+      </x:c>
+      <x:c r="U207" s="23" t="str">
+        <x:v>공식 상품 상세에 1,170 TRY(KDV 포함).</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="208" ht="36" customHeight="1">
+      <x:c r="A208" t="str">
+        <x:v>IST-SV-002</x:v>
+      </x:c>
+      <x:c r="B208" t="str">
+        <x:v>튀르키예</x:v>
+      </x:c>
+      <x:c r="C208" t="str">
+        <x:v>이스탄불</x:v>
+      </x:c>
+      <x:c r="D208" t="str">
+        <x:v>기념품</x:v>
+      </x:c>
+      <x:c r="E208" t="str">
+        <x:v>식품</x:v>
+      </x:c>
+      <x:c r="F208" t="str">
+        <x:v>Kurukahveci Mehmet Efendi Türk Kahvesi 5×100g</x:v>
+      </x:c>
+      <x:c r="G208" t="str">
+        <x:v>Kurukahveci Mehmet Efendi Turkish Coffee, 5×100 g</x:v>
+      </x:c>
+      <x:c r="H208" s="55" t="n">
+        <x:v>465</x:v>
+      </x:c>
+      <x:c r="I208" s="55" t="n">
+        <x:v>465</x:v>
+      </x:c>
+      <x:c r="J208" t="str">
+        <x:v>TRY</x:v>
+      </x:c>
+      <x:c r="K208" t="str">
+        <x:v>1상자 500g</x:v>
+      </x:c>
+      <x:c r="L208" t="str">
+        <x:v>고정형</x:v>
+      </x:c>
+      <x:c r="M208" t="str">
+        <x:v>일반</x:v>
+      </x:c>
+      <x:c r="N208" t="str">
+        <x:v>A 공식</x:v>
+      </x:c>
+      <x:c r="O208" t="str">
+        <x:v>예</x:v>
+      </x:c>
+      <x:c r="P208" t="str">
+        <x:v>확정 1차</x:v>
+      </x:c>
+      <x:c r="Q208" s="51" t="n">
+        <x:v>46298</x:v>
+      </x:c>
+      <x:c r="R208" t="str">
+        <x:v>2026-10-03 확인</x:v>
+      </x:c>
+      <x:c r="S208" t="str">
+        <x:v>Kurukahveci Mehmet Efendi</x:v>
+      </x:c>
+      <x:c r="T208" t="str">
+        <x:v>https://online.mehmetefendi.com/turk-kahvesi-5x100g</x:v>
+      </x:c>
+      <x:c r="U208" s="23" t="str">
+        <x:v>공식 상품 상세에 465 TRY(KDV 포함).</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="209" ht="36" customHeight="1">
+      <x:c r="A209" t="str">
+        <x:v>IST-SV-003</x:v>
+      </x:c>
+      <x:c r="B209" t="str">
+        <x:v>튀르키예</x:v>
+      </x:c>
+      <x:c r="C209" t="str">
+        <x:v>이스탄불</x:v>
+      </x:c>
+      <x:c r="D209" t="str">
+        <x:v>기념품</x:v>
+      </x:c>
+      <x:c r="E209" t="str">
+        <x:v>잡화</x:v>
+      </x:c>
+      <x:c r="F209" t="str">
+        <x:v>Kurukahveci Mehmet Efendi 레트로 자석 Kahve İçen Yorulmaz</x:v>
+      </x:c>
+      <x:c r="G209" t="str">
+        <x:v>Kurukahveci Mehmet Efendi Retro Magnet, Kahve İçen Yorulmaz</x:v>
+      </x:c>
+      <x:c r="H209" s="55" t="n">
+        <x:v>55</x:v>
+      </x:c>
+      <x:c r="I209" s="55" t="n">
+        <x:v>55</x:v>
+      </x:c>
+      <x:c r="J209" t="str">
+        <x:v>TRY</x:v>
+      </x:c>
+      <x:c r="K209" t="str">
+        <x:v>1개</x:v>
+      </x:c>
+      <x:c r="L209" t="str">
+        <x:v>고정형</x:v>
+      </x:c>
+      <x:c r="M209" t="str">
+        <x:v>일반</x:v>
+      </x:c>
+      <x:c r="N209" t="str">
+        <x:v>A 공식</x:v>
+      </x:c>
+      <x:c r="O209" t="str">
+        <x:v>예</x:v>
+      </x:c>
+      <x:c r="P209" t="str">
+        <x:v>확정 1차</x:v>
+      </x:c>
+      <x:c r="Q209" s="51" t="n">
+        <x:v>46298</x:v>
+      </x:c>
+      <x:c r="R209" t="str">
+        <x:v>2026-10-03 확인</x:v>
+      </x:c>
+      <x:c r="S209" t="str">
+        <x:v>Kurukahveci Mehmet Efendi</x:v>
+      </x:c>
+      <x:c r="T209" t="str">
+        <x:v>https://online.mehmetefendi.com/retro-koleksiyon-magnet-kahve-icen-yorulmaz</x:v>
+      </x:c>
+      <x:c r="U209" s="23" t="str">
+        <x:v>공식 상품 상세에 55 TRY(KDV 포함), 크기 8.5×5.5cm.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="210" ht="36" customHeight="1">
+      <x:c r="A210" t="str">
+        <x:v>IST-AT-001</x:v>
+      </x:c>
+      <x:c r="B210" t="str">
+        <x:v>튀르키예</x:v>
+      </x:c>
+      <x:c r="C210" t="str">
+        <x:v>이스탄불</x:v>
+      </x:c>
+      <x:c r="D210" t="str">
+        <x:v>관광</x:v>
+      </x:c>
+      <x:c r="E210" t="str">
+        <x:v>궁전</x:v>
+      </x:c>
+      <x:c r="F210" t="str">
+        <x:v>Topkapı Sarayı 복합 입장권 외국인 성인</x:v>
+      </x:c>
+      <x:c r="G210" t="str">
+        <x:v>Topkapi Palace Combined Admission, Foreign Adult</x:v>
+      </x:c>
+      <x:c r="H210" s="55" t="n">
+        <x:v>2750</x:v>
+      </x:c>
+      <x:c r="I210" s="55" t="n">
+        <x:v>2750</x:v>
+      </x:c>
+      <x:c r="J210" t="str">
+        <x:v>TRY</x:v>
+      </x:c>
+      <x:c r="K210" t="str">
+        <x:v>외국인 1인</x:v>
+      </x:c>
+      <x:c r="L210" t="str">
+        <x:v>고정형</x:v>
+      </x:c>
+      <x:c r="M210" t="str">
+        <x:v>외국인 성인</x:v>
+      </x:c>
+      <x:c r="N210" t="str">
+        <x:v>B 공공</x:v>
+      </x:c>
+      <x:c r="O210" t="str">
+        <x:v>예</x:v>
+      </x:c>
+      <x:c r="P210" t="str">
+        <x:v>확정 1차</x:v>
+      </x:c>
+      <x:c r="Q210" s="51" t="n">
+        <x:v>46298</x:v>
+      </x:c>
+      <x:c r="R210" t="str">
+        <x:v>2026-10-03 확인</x:v>
+      </x:c>
+      <x:c r="S210" t="str">
+        <x:v>Millî Saraylar</x:v>
+      </x:c>
+      <x:c r="T210" t="str">
+        <x:v>https://www.millisaraylar.gov.tr/Lokasyon/2/Topkapi-Sarayi?culture=en</x:v>
+      </x:c>
+      <x:c r="U210" s="23" t="str">
+        <x:v>외국인 복합 입장권(Topkapı + Hagia Irene + Harem) 2,750 TRY.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="211" ht="36" customHeight="1">
+      <x:c r="A211" t="str">
+        <x:v>IST-AT-002</x:v>
+      </x:c>
+      <x:c r="B211" t="str">
+        <x:v>튀르키예</x:v>
+      </x:c>
+      <x:c r="C211" t="str">
+        <x:v>이스탄불</x:v>
+      </x:c>
+      <x:c r="D211" t="str">
+        <x:v>관광</x:v>
+      </x:c>
+      <x:c r="E211" t="str">
+        <x:v>궁전</x:v>
+      </x:c>
+      <x:c r="F211" t="str">
+        <x:v>Dolmabahçe Sarayı 통합 입장권 외국인 성인</x:v>
+      </x:c>
+      <x:c r="G211" t="str">
+        <x:v>Dolmabahce Palace Combined Admission, Foreign Adult</x:v>
+      </x:c>
+      <x:c r="H211" s="55" t="n">
+        <x:v>2000</x:v>
+      </x:c>
+      <x:c r="I211" s="55" t="n">
+        <x:v>2000</x:v>
+      </x:c>
+      <x:c r="J211" t="str">
+        <x:v>TRY</x:v>
+      </x:c>
+      <x:c r="K211" t="str">
+        <x:v>외국인 1인</x:v>
+      </x:c>
+      <x:c r="L211" t="str">
+        <x:v>고정형</x:v>
+      </x:c>
+      <x:c r="M211" t="str">
+        <x:v>외국인 성인</x:v>
+      </x:c>
+      <x:c r="N211" t="str">
+        <x:v>B 공공</x:v>
+      </x:c>
+      <x:c r="O211" t="str">
+        <x:v>예</x:v>
+      </x:c>
+      <x:c r="P211" t="str">
+        <x:v>확정 1차</x:v>
+      </x:c>
+      <x:c r="Q211" s="51" t="n">
+        <x:v>46298</x:v>
+      </x:c>
+      <x:c r="R211" t="str">
+        <x:v>2026-10-03 확인</x:v>
+      </x:c>
+      <x:c r="S211" t="str">
+        <x:v>Millî Saraylar</x:v>
+      </x:c>
+      <x:c r="T211" t="str">
+        <x:v>https://millisaraylar.gov.tr/Lokasyon/3/Dolmabahce-Sarayi</x:v>
+      </x:c>
+      <x:c r="U211" s="23" t="str">
+        <x:v>외국인 Selamlık·Harem·Resim Müzesi 통합권 2,000 TRY.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="212" ht="36" customHeight="1">
+      <x:c r="A212" t="str">
+        <x:v>IST-AT-003</x:v>
+      </x:c>
+      <x:c r="B212" t="str">
+        <x:v>튀르키예</x:v>
+      </x:c>
+      <x:c r="C212" t="str">
+        <x:v>이스탄불</x:v>
+      </x:c>
+      <x:c r="D212" t="str">
+        <x:v>관광</x:v>
+      </x:c>
+      <x:c r="E212" t="str">
+        <x:v>궁전</x:v>
+      </x:c>
+      <x:c r="F212" t="str">
+        <x:v>Beylerbeyi Sarayı 외국인 성인 입장</x:v>
+      </x:c>
+      <x:c r="G212" t="str">
+        <x:v>Beylerbeyi Palace Admission, Foreign Adult</x:v>
+      </x:c>
+      <x:c r="H212" s="55" t="n">
+        <x:v>800</x:v>
+      </x:c>
+      <x:c r="I212" s="55" t="n">
+        <x:v>800</x:v>
+      </x:c>
+      <x:c r="J212" t="str">
+        <x:v>TRY</x:v>
+      </x:c>
+      <x:c r="K212" t="str">
+        <x:v>외국인 1인</x:v>
+      </x:c>
+      <x:c r="L212" t="str">
+        <x:v>고정형</x:v>
+      </x:c>
+      <x:c r="M212" t="str">
+        <x:v>외국인 성인</x:v>
+      </x:c>
+      <x:c r="N212" t="str">
+        <x:v>B 공공</x:v>
+      </x:c>
+      <x:c r="O212" t="str">
+        <x:v>예</x:v>
+      </x:c>
+      <x:c r="P212" t="str">
+        <x:v>확정 1차</x:v>
+      </x:c>
+      <x:c r="Q212" s="51" t="n">
+        <x:v>46298</x:v>
+      </x:c>
+      <x:c r="R212" t="str">
+        <x:v>2026-10-03 확인</x:v>
+      </x:c>
+      <x:c r="S212" t="str">
+        <x:v>Millî Saraylar</x:v>
+      </x:c>
+      <x:c r="T212" t="str">
+        <x:v>https://millisaraylar.gov.tr/Lokasyon/4/Beylerbeyi-Sarayi</x:v>
+      </x:c>
+      <x:c r="U212" s="23" t="str">
+        <x:v>공식 외국인 방문객 입장료 800 TRY.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="213" ht="36" customHeight="1">
+      <x:c r="A213" t="str">
+        <x:v>IST-AT-004</x:v>
+      </x:c>
+      <x:c r="B213" t="str">
+        <x:v>튀르키예</x:v>
+      </x:c>
+      <x:c r="C213" t="str">
+        <x:v>이스탄불</x:v>
+      </x:c>
+      <x:c r="D213" t="str">
+        <x:v>관광</x:v>
+      </x:c>
+      <x:c r="E213" t="str">
+        <x:v>궁전</x:v>
+      </x:c>
+      <x:c r="F213" t="str">
+        <x:v>Yıldız Sarayı 외국인 성인 입장</x:v>
+      </x:c>
+      <x:c r="G213" t="str">
+        <x:v>Yildiz Palace Admission, Foreign Adult</x:v>
+      </x:c>
+      <x:c r="H213" s="55" t="n">
+        <x:v>900</x:v>
+      </x:c>
+      <x:c r="I213" s="55" t="n">
+        <x:v>900</x:v>
+      </x:c>
+      <x:c r="J213" t="str">
+        <x:v>TRY</x:v>
+      </x:c>
+      <x:c r="K213" t="str">
+        <x:v>외국인 1인</x:v>
+      </x:c>
+      <x:c r="L213" t="str">
+        <x:v>고정형</x:v>
+      </x:c>
+      <x:c r="M213" t="str">
+        <x:v>외국인 성인</x:v>
+      </x:c>
+      <x:c r="N213" t="str">
+        <x:v>B 공공</x:v>
+      </x:c>
+      <x:c r="O213" t="str">
+        <x:v>예</x:v>
+      </x:c>
+      <x:c r="P213" t="str">
+        <x:v>확정 1차</x:v>
+      </x:c>
+      <x:c r="Q213" s="51" t="n">
+        <x:v>46298</x:v>
+      </x:c>
+      <x:c r="R213" t="str">
+        <x:v>2026-10-03 확인</x:v>
+      </x:c>
+      <x:c r="S213" t="str">
+        <x:v>Millî Saraylar</x:v>
+      </x:c>
+      <x:c r="T213" t="str">
+        <x:v>https://www.millisaraylar.gov.tr/Lokasyon/5/Yildiz-Sarayi?culture=en</x:v>
+      </x:c>
+      <x:c r="U213" s="23" t="str">
+        <x:v>공식 외국인 방문객 입장료 900 TRY.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="214" ht="36" customHeight="1">
+      <x:c r="A214" t="str">
+        <x:v>IST-AT-005</x:v>
+      </x:c>
+      <x:c r="B214" t="str">
+        <x:v>튀르키예</x:v>
+      </x:c>
+      <x:c r="C214" t="str">
+        <x:v>이스탄불</x:v>
+      </x:c>
+      <x:c r="D214" t="str">
+        <x:v>관광</x:v>
+      </x:c>
+      <x:c r="E214" t="str">
+        <x:v>랜드마크</x:v>
+      </x:c>
+      <x:c r="F214" t="str">
+        <x:v>Galata Kulesi 외국인 입장권</x:v>
+      </x:c>
+      <x:c r="G214" t="str">
+        <x:v>Galata Tower Museum Admission</x:v>
+      </x:c>
+      <x:c r="H214" s="55" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="I214" s="55" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="J214" t="str">
+        <x:v>EUR</x:v>
+      </x:c>
+      <x:c r="K214" t="str">
+        <x:v>외국인 1인</x:v>
+      </x:c>
+      <x:c r="L214" t="str">
+        <x:v>고정형</x:v>
+      </x:c>
+      <x:c r="M214" t="str">
+        <x:v>외국인 성인</x:v>
+      </x:c>
+      <x:c r="N214" t="str">
+        <x:v>B 공공</x:v>
+      </x:c>
+      <x:c r="O214" t="str">
+        <x:v>예</x:v>
+      </x:c>
+      <x:c r="P214" t="str">
+        <x:v>확정 1차</x:v>
+      </x:c>
+      <x:c r="Q214" s="51" t="n">
+        <x:v>46298</x:v>
+      </x:c>
+      <x:c r="R214" t="str">
+        <x:v>2026-10-03 확인</x:v>
+      </x:c>
+      <x:c r="S214" t="str">
+        <x:v>T.C. Kültür ve Turizm Bakanlığı / Müze.gov.tr</x:v>
+      </x:c>
+      <x:c r="T214" t="str">
+        <x:v>https://muze.gov.tr/urun-ekle?catalogNo=WEB-CUM01-87-009</x:v>
+      </x:c>
+      <x:c r="U214" s="23" t="str">
+        <x:v>문화관광부 공식 전자티켓 상품 가격 30 EUR.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="215" ht="36" customHeight="1">
+      <x:c r="A215" t="str">
+        <x:v>IST-AT-006</x:v>
+      </x:c>
+      <x:c r="B215" t="str">
+        <x:v>튀르키예</x:v>
+      </x:c>
+      <x:c r="C215" t="str">
+        <x:v>이스탄불</x:v>
+      </x:c>
+      <x:c r="D215" t="str">
+        <x:v>관광</x:v>
+      </x:c>
+      <x:c r="E215" t="str">
+        <x:v>랜드마크</x:v>
+      </x:c>
+      <x:c r="F215" t="str">
+        <x:v>Kız Kulesi 외국인 입장권</x:v>
+      </x:c>
+      <x:c r="G215" t="str">
+        <x:v>Maiden's Tower Admission</x:v>
+      </x:c>
+      <x:c r="H215" s="55" t="n">
+        <x:v>27</x:v>
+      </x:c>
+      <x:c r="I215" s="55" t="n">
+        <x:v>27</x:v>
+      </x:c>
+      <x:c r="J215" t="str">
+        <x:v>EUR</x:v>
+      </x:c>
+      <x:c r="K215" t="str">
+        <x:v>외국인 1인</x:v>
+      </x:c>
+      <x:c r="L215" t="str">
+        <x:v>고정형</x:v>
+      </x:c>
+      <x:c r="M215" t="str">
+        <x:v>외국인 성인</x:v>
+      </x:c>
+      <x:c r="N215" t="str">
+        <x:v>B 공공</x:v>
+      </x:c>
+      <x:c r="O215" t="str">
+        <x:v>예</x:v>
+      </x:c>
+      <x:c r="P215" t="str">
+        <x:v>확정 1차</x:v>
+      </x:c>
+      <x:c r="Q215" s="51" t="n">
+        <x:v>46298</x:v>
+      </x:c>
+      <x:c r="R215" t="str">
+        <x:v>2026-10-03 확인</x:v>
+      </x:c>
+      <x:c r="S215" t="str">
+        <x:v>T.C. Kültür ve Turizm Bakanlığı / Müze.gov.tr</x:v>
+      </x:c>
+      <x:c r="T215" t="str">
+        <x:v>https://muze.gov.tr/urun-ekle?catalogNo=WEB-CUM01-87-009</x:v>
+      </x:c>
+      <x:c r="U215" s="23" t="str">
+        <x:v>문화관광부 공식 전자티켓 상품 가격 27 EUR.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="216" ht="36" customHeight="1">
+      <x:c r="A216" t="str">
+        <x:v>IST-AT-007</x:v>
+      </x:c>
+      <x:c r="B216" t="str">
+        <x:v>튀르키예</x:v>
+      </x:c>
+      <x:c r="C216" t="str">
+        <x:v>이스탄불</x:v>
+      </x:c>
+      <x:c r="D216" t="str">
+        <x:v>관광</x:v>
+      </x:c>
+      <x:c r="E216" t="str">
+        <x:v>박물관</x:v>
+      </x:c>
+      <x:c r="F216" t="str">
+        <x:v>İstanbul Arkeoloji Müzeleri 외국인 입장권</x:v>
+      </x:c>
+      <x:c r="G216" t="str">
+        <x:v>Istanbul Archaeological Museums Admission</x:v>
+      </x:c>
+      <x:c r="H216" s="55" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="I216" s="55" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="J216" t="str">
+        <x:v>EUR</x:v>
+      </x:c>
+      <x:c r="K216" t="str">
+        <x:v>외국인 1인</x:v>
+      </x:c>
+      <x:c r="L216" t="str">
+        <x:v>고정형</x:v>
+      </x:c>
+      <x:c r="M216" t="str">
+        <x:v>외국인 성인</x:v>
+      </x:c>
+      <x:c r="N216" t="str">
+        <x:v>B 공공</x:v>
+      </x:c>
+      <x:c r="O216" t="str">
+        <x:v>예</x:v>
+      </x:c>
+      <x:c r="P216" t="str">
+        <x:v>확정 1차</x:v>
+      </x:c>
+      <x:c r="Q216" s="51" t="n">
+        <x:v>46298</x:v>
+      </x:c>
+      <x:c r="R216" t="str">
+        <x:v>2026-10-03 확인</x:v>
+      </x:c>
+      <x:c r="S216" t="str">
+        <x:v>T.C. Kültür ve Turizm Bakanlığı / Müze.gov.tr</x:v>
+      </x:c>
+      <x:c r="T216" t="str">
+        <x:v>https://muze.gov.tr/urun-ekle?catalogNo=WEB-CUM01-87-009</x:v>
+      </x:c>
+      <x:c r="U216" s="23" t="str">
+        <x:v>문화관광부 공식 전자티켓 상품 가격 15 EUR.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="217" ht="36" customHeight="1">
+      <x:c r="A217" t="str">
+        <x:v>IST-AT-008</x:v>
+      </x:c>
+      <x:c r="B217" t="str">
+        <x:v>튀르키예</x:v>
+      </x:c>
+      <x:c r="C217" t="str">
+        <x:v>이스탄불</x:v>
+      </x:c>
+      <x:c r="D217" t="str">
+        <x:v>관광</x:v>
+      </x:c>
+      <x:c r="E217" t="str">
+        <x:v>박물관</x:v>
+      </x:c>
+      <x:c r="F217" t="str">
+        <x:v>İstanbul Modern 일반 방문객 입장권</x:v>
+      </x:c>
+      <x:c r="G217" t="str">
+        <x:v>Istanbul Modern Regular Admission</x:v>
+      </x:c>
+      <x:c r="H217" s="55" t="n">
+        <x:v>1000</x:v>
+      </x:c>
+      <x:c r="I217" s="55" t="n">
+        <x:v>1000</x:v>
+      </x:c>
+      <x:c r="J217" t="str">
+        <x:v>TRY</x:v>
+      </x:c>
+      <x:c r="K217" t="str">
+        <x:v>일반 1인</x:v>
+      </x:c>
+      <x:c r="L217" t="str">
+        <x:v>고정형</x:v>
+      </x:c>
+      <x:c r="M217" t="str">
+        <x:v>비거주자 성인</x:v>
+      </x:c>
+      <x:c r="N217" t="str">
+        <x:v>A 공식</x:v>
+      </x:c>
+      <x:c r="O217" t="str">
+        <x:v>예</x:v>
+      </x:c>
+      <x:c r="P217" t="str">
+        <x:v>확정 1차</x:v>
+      </x:c>
+      <x:c r="Q217" s="51" t="n">
+        <x:v>46298</x:v>
+      </x:c>
+      <x:c r="R217" t="str">
+        <x:v>2026-10-03 확인</x:v>
+      </x:c>
+      <x:c r="S217" t="str">
+        <x:v>İstanbul Modern</x:v>
+      </x:c>
+      <x:c r="T217" t="str">
+        <x:v>https://www.istanbulmodern.org/en/visit/museum</x:v>
+      </x:c>
+      <x:c r="U217" s="23" t="str">
+        <x:v>미술관 공식 요금표 일반 입장 1,000 TRY, Türkiye 거주자 일반권은 별도 600 TRY.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="218" ht="36" customHeight="1">
+      <x:c r="A218" t="str">
+        <x:v>IST-AT-009</x:v>
+      </x:c>
+      <x:c r="B218" t="str">
+        <x:v>튀르키예</x:v>
+      </x:c>
+      <x:c r="C218" t="str">
+        <x:v>이스탄불</x:v>
+      </x:c>
+      <x:c r="D218" t="str">
+        <x:v>관광</x:v>
+      </x:c>
+      <x:c r="E218" t="str">
+        <x:v>궁전</x:v>
+      </x:c>
+      <x:c r="F218" t="str">
+        <x:v>Topkapı Sarayı 0–6세 무료 입장</x:v>
+      </x:c>
+      <x:c r="G218" t="str">
+        <x:v>Topkapi Palace Free Admission, Ages 0–6</x:v>
+      </x:c>
+      <x:c r="H218" s="55" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I218" s="55" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J218" t="str">
+        <x:v>TRY</x:v>
+      </x:c>
+      <x:c r="K218" t="str">
+        <x:v>아동 1인</x:v>
+      </x:c>
+      <x:c r="L218" t="str">
+        <x:v>일정/대상형</x:v>
+      </x:c>
+      <x:c r="M218" t="str">
+        <x:v>외국인 만 0~6세</x:v>
+      </x:c>
+      <x:c r="N218" t="str">
+        <x:v>B 공공</x:v>
+      </x:c>
+      <x:c r="O218" t="str">
+        <x:v>예</x:v>
+      </x:c>
+      <x:c r="P218" t="str">
+        <x:v>확정 1차</x:v>
+      </x:c>
+      <x:c r="Q218" s="51" t="n">
+        <x:v>46298</x:v>
+      </x:c>
+      <x:c r="R218" t="str">
+        <x:v>2026-10-03 확인</x:v>
+      </x:c>
+      <x:c r="S218" t="str">
+        <x:v>Millî Saraylar</x:v>
+      </x:c>
+      <x:c r="T218" t="str">
+        <x:v>https://www.millisaraylar.gov.tr/Lokasyon/2/Topkapi-Sarayi?culture=en</x:v>
+      </x:c>
+      <x:c r="U218" s="23" t="str">
+        <x:v>공식 안내에서 국내·외 방문객 0–6세 무료 명시.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="219" ht="36" customHeight="1">
+      <x:c r="A219" t="str">
+        <x:v>IST-AT-010</x:v>
+      </x:c>
+      <x:c r="B219" t="str">
+        <x:v>튀르키예</x:v>
+      </x:c>
+      <x:c r="C219" t="str">
+        <x:v>이스탄불</x:v>
+      </x:c>
+      <x:c r="D219" t="str">
+        <x:v>관광</x:v>
+      </x:c>
+      <x:c r="E219" t="str">
+        <x:v>궁전</x:v>
+      </x:c>
+      <x:c r="F219" t="str">
+        <x:v>Dolmabahçe Sarayı 0–6세 무료 입장</x:v>
+      </x:c>
+      <x:c r="G219" t="str">
+        <x:v>Dolmabahce Palace Free Admission, Ages 0–6</x:v>
+      </x:c>
+      <x:c r="H219" s="55" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I219" s="55" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J219" t="str">
+        <x:v>TRY</x:v>
+      </x:c>
+      <x:c r="K219" t="str">
+        <x:v>아동 1인</x:v>
+      </x:c>
+      <x:c r="L219" t="str">
+        <x:v>일정/대상형</x:v>
+      </x:c>
+      <x:c r="M219" t="str">
+        <x:v>외국인 만 0~6세</x:v>
+      </x:c>
+      <x:c r="N219" t="str">
+        <x:v>B 공공</x:v>
+      </x:c>
+      <x:c r="O219" t="str">
+        <x:v>예</x:v>
+      </x:c>
+      <x:c r="P219" t="str">
+        <x:v>확정 1차</x:v>
+      </x:c>
+      <x:c r="Q219" s="51" t="n">
+        <x:v>46298</x:v>
+      </x:c>
+      <x:c r="R219" t="str">
+        <x:v>2026-10-03 확인</x:v>
+      </x:c>
+      <x:c r="S219" t="str">
+        <x:v>Millî Saraylar</x:v>
+      </x:c>
+      <x:c r="T219" t="str">
+        <x:v>https://millisaraylar.gov.tr/Lokasyon/3/Dolmabahce-Sarayi</x:v>
+      </x:c>
+      <x:c r="U219" s="23" t="str">
+        <x:v>공식 안내에서 국내·외 방문객 0–6세 무료 명시.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="220" ht="36" customHeight="1">
+      <x:c r="A220" t="str">
+        <x:v>IST-AT-011</x:v>
+      </x:c>
+      <x:c r="B220" t="str">
+        <x:v>튀르키예</x:v>
+      </x:c>
+      <x:c r="C220" t="str">
+        <x:v>이스탄불</x:v>
+      </x:c>
+      <x:c r="D220" t="str">
+        <x:v>관광</x:v>
+      </x:c>
+      <x:c r="E220" t="str">
+        <x:v>궁전</x:v>
+      </x:c>
+      <x:c r="F220" t="str">
+        <x:v>Beylerbeyi Sarayı 0–6세 무료 입장</x:v>
+      </x:c>
+      <x:c r="G220" t="str">
+        <x:v>Beylerbeyi Palace Free Admission, Ages 0–6</x:v>
+      </x:c>
+      <x:c r="H220" s="55" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I220" s="55" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J220" t="str">
+        <x:v>TRY</x:v>
+      </x:c>
+      <x:c r="K220" t="str">
+        <x:v>아동 1인</x:v>
+      </x:c>
+      <x:c r="L220" t="str">
+        <x:v>일정/대상형</x:v>
+      </x:c>
+      <x:c r="M220" t="str">
+        <x:v>외국인 만 0~6세</x:v>
+      </x:c>
+      <x:c r="N220" t="str">
+        <x:v>B 공공</x:v>
+      </x:c>
+      <x:c r="O220" t="str">
+        <x:v>예</x:v>
+      </x:c>
+      <x:c r="P220" t="str">
+        <x:v>확정 1차</x:v>
+      </x:c>
+      <x:c r="Q220" s="51" t="n">
+        <x:v>46298</x:v>
+      </x:c>
+      <x:c r="R220" t="str">
+        <x:v>2026-10-03 확인</x:v>
+      </x:c>
+      <x:c r="S220" t="str">
+        <x:v>Millî Saraylar</x:v>
+      </x:c>
+      <x:c r="T220" t="str">
+        <x:v>https://millisaraylar.gov.tr/Lokasyon/4/Beylerbeyi-Sarayi</x:v>
+      </x:c>
+      <x:c r="U220" s="23" t="str">
+        <x:v>공식 안내에서 국내·외 방문객 0–6세 무료 명시.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="221" ht="36" customHeight="1">
+      <x:c r="A221" t="str">
+        <x:v>IST-AT-012</x:v>
+      </x:c>
+      <x:c r="B221" t="str">
+        <x:v>튀르키예</x:v>
+      </x:c>
+      <x:c r="C221" t="str">
+        <x:v>이스탄불</x:v>
+      </x:c>
+      <x:c r="D221" t="str">
+        <x:v>관광</x:v>
+      </x:c>
+      <x:c r="E221" t="str">
+        <x:v>궁전</x:v>
+      </x:c>
+      <x:c r="F221" t="str">
+        <x:v>Yıldız Sarayı 0–6세 무료 입장</x:v>
+      </x:c>
+      <x:c r="G221" t="str">
+        <x:v>Yildiz Palace Free Admission, Ages 0–6</x:v>
+      </x:c>
+      <x:c r="H221" s="55" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I221" s="55" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J221" t="str">
+        <x:v>TRY</x:v>
+      </x:c>
+      <x:c r="K221" t="str">
+        <x:v>아동 1인</x:v>
+      </x:c>
+      <x:c r="L221" t="str">
+        <x:v>일정/대상형</x:v>
+      </x:c>
+      <x:c r="M221" t="str">
+        <x:v>외국인 만 0~6세</x:v>
+      </x:c>
+      <x:c r="N221" t="str">
+        <x:v>B 공공</x:v>
+      </x:c>
+      <x:c r="O221" t="str">
+        <x:v>예</x:v>
+      </x:c>
+      <x:c r="P221" t="str">
+        <x:v>확정 1차</x:v>
+      </x:c>
+      <x:c r="Q221" s="51" t="n">
+        <x:v>46298</x:v>
+      </x:c>
+      <x:c r="R221" t="str">
+        <x:v>2026-10-03 확인</x:v>
+      </x:c>
+      <x:c r="S221" t="str">
+        <x:v>Millî Saraylar</x:v>
+      </x:c>
+      <x:c r="T221" t="str">
+        <x:v>https://www.millisaraylar.gov.tr/Lokasyon/5/Yildiz-Sarayi?culture=en</x:v>
+      </x:c>
+      <x:c r="U221" s="23" t="str">
+        <x:v>공식 안내에서 국내·외 방문객 0–6세 무료 명시.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="222" ht="36" customHeight="1">
+      <x:c r="A222" t="str">
+        <x:v>IST-AT-013</x:v>
+      </x:c>
+      <x:c r="B222" t="str">
+        <x:v>튀르키예</x:v>
+      </x:c>
+      <x:c r="C222" t="str">
+        <x:v>이스탄불</x:v>
+      </x:c>
+      <x:c r="D222" t="str">
+        <x:v>관광</x:v>
+      </x:c>
+      <x:c r="E222" t="str">
+        <x:v>박물관</x:v>
+      </x:c>
+      <x:c r="F222" t="str">
+        <x:v>İstanbul Modern 12세 미만 무료 입장</x:v>
+      </x:c>
+      <x:c r="G222" t="str">
+        <x:v>Istanbul Modern Free Admission, Under 12</x:v>
+      </x:c>
+      <x:c r="H222" s="55" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I222" s="55" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J222" t="str">
+        <x:v>TRY</x:v>
+      </x:c>
+      <x:c r="K222" t="str">
+        <x:v>아동 1인</x:v>
+      </x:c>
+      <x:c r="L222" t="str">
+        <x:v>일정/대상형</x:v>
+      </x:c>
+      <x:c r="M222" t="str">
+        <x:v>만 12세 미만</x:v>
+      </x:c>
+      <x:c r="N222" t="str">
+        <x:v>A 공식</x:v>
+      </x:c>
+      <x:c r="O222" t="str">
+        <x:v>예</x:v>
+      </x:c>
+      <x:c r="P222" t="str">
+        <x:v>확정 1차</x:v>
+      </x:c>
+      <x:c r="Q222" s="51" t="n">
+        <x:v>46298</x:v>
+      </x:c>
+      <x:c r="R222" t="str">
+        <x:v>2026-10-03 확인</x:v>
+      </x:c>
+      <x:c r="S222" t="str">
+        <x:v>İstanbul Modern</x:v>
+      </x:c>
+      <x:c r="T222" t="str">
+        <x:v>https://www.istanbulmodern.org/en/visit/museum</x:v>
+      </x:c>
+      <x:c r="U222" s="23" t="str">
+        <x:v>미술관 공식 안내에서 12세 미만 무료 명시.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:U1"/>
@@ -13980,7 +16060,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra1d50a7722c64e50"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re02919e1fc064476"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -15428,6 +17508,171 @@
         <x:v>공식 지점별 가격 확보</x:v>
       </x:c>
     </x:row>
+    <x:row r="45" ht="44" customHeight="1">
+      <x:c r="A45" s="23" t="str">
+        <x:v>튀르키예</x:v>
+      </x:c>
+      <x:c r="B45" s="23" t="str">
+        <x:v>이스탄불</x:v>
+      </x:c>
+      <x:c r="C45" s="23" t="str">
+        <x:v>되네르 케밥</x:v>
+      </x:c>
+      <x:c r="D45" s="23" t="str">
+        <x:v>Döner kebab</x:v>
+      </x:c>
+      <x:c r="E45" s="23" t="str">
+        <x:v>이스탄불의 대표적인 길거리 음식으로 소개되며, 고기와 채소를 빵이나 라바시에 담아 먹는다.</x:v>
+      </x:c>
+      <x:c r="F45" s="23" t="str">
+        <x:v>미조사</x:v>
+      </x:c>
+      <x:c r="G45" s="23"/>
+      <x:c r="H45" s="23" t="str">
+        <x:v>대기</x:v>
+      </x:c>
+      <x:c r="I45" s="23" t="str">
+        <x:v>GoTürkiye</x:v>
+      </x:c>
+      <x:c r="J45" s="23" t="str">
+        <x:v>https://goturkiye.com/branding/the-10-most-popular-street-foods-of-istanbul</x:v>
+      </x:c>
+      <x:c r="K45" s="23" t="str">
+        <x:v>관광청 음식 추천만 기록. 공식 판매 가격 표본은 별도로 확인하지 않아 가격대는 입력하지 않음.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="46" ht="44" customHeight="1">
+      <x:c r="A46" s="23" t="str">
+        <x:v>튀르키예</x:v>
+      </x:c>
+      <x:c r="B46" s="23" t="str">
+        <x:v>이스탄불</x:v>
+      </x:c>
+      <x:c r="C46" s="23" t="str">
+        <x:v>시미트</x:v>
+      </x:c>
+      <x:c r="D46" s="23" t="str">
+        <x:v>Simit</x:v>
+      </x:c>
+      <x:c r="E46" s="23" t="str">
+        <x:v>참깨를 얹은 고리 모양 빵으로, 이스탄불의 아침 식사와 길거리 간식으로 소개된다.</x:v>
+      </x:c>
+      <x:c r="F46" s="23" t="str">
+        <x:v>미조사</x:v>
+      </x:c>
+      <x:c r="G46" s="23"/>
+      <x:c r="H46" s="23" t="str">
+        <x:v>대기</x:v>
+      </x:c>
+      <x:c r="I46" s="23" t="str">
+        <x:v>GoTürkiye</x:v>
+      </x:c>
+      <x:c r="J46" s="23" t="str">
+        <x:v>https://goturkiye.com/branding/the-10-most-popular-street-foods-of-istanbul</x:v>
+      </x:c>
+      <x:c r="K46" s="23" t="str">
+        <x:v>관광청 음식 추천만 기록. 공식 판매 가격 표본은 별도로 확인하지 않아 가격대는 입력하지 않음.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="47" ht="44" customHeight="1">
+      <x:c r="A47" s="23" t="str">
+        <x:v>튀르키예</x:v>
+      </x:c>
+      <x:c r="B47" s="23" t="str">
+        <x:v>이스탄불</x:v>
+      </x:c>
+      <x:c r="C47" s="23" t="str">
+        <x:v>코코레치</x:v>
+      </x:c>
+      <x:c r="D47" s="23" t="str">
+        <x:v>Kokoreç</x:v>
+      </x:c>
+      <x:c r="E47" s="23" t="str">
+        <x:v>양 내장을 향신료와 함께 구운 뒤 샌드위치 형태로 먹는 이스탄불 길거리 음식으로 소개된다.</x:v>
+      </x:c>
+      <x:c r="F47" s="23" t="str">
+        <x:v>미조사</x:v>
+      </x:c>
+      <x:c r="G47" s="23"/>
+      <x:c r="H47" s="23" t="str">
+        <x:v>대기</x:v>
+      </x:c>
+      <x:c r="I47" s="23" t="str">
+        <x:v>GoTürkiye</x:v>
+      </x:c>
+      <x:c r="J47" s="23" t="str">
+        <x:v>https://goturkiye.com/branding/the-10-most-popular-street-foods-of-istanbul</x:v>
+      </x:c>
+      <x:c r="K47" s="23" t="str">
+        <x:v>관광청 음식 추천만 기록. 공식 판매 가격 표본은 별도로 확인하지 않아 가격대는 입력하지 않음.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="48" ht="44" customHeight="1">
+      <x:c r="A48" s="23" t="str">
+        <x:v>튀르키예</x:v>
+      </x:c>
+      <x:c r="B48" s="23" t="str">
+        <x:v>이스탄불</x:v>
+      </x:c>
+      <x:c r="C48" s="23" t="str">
+        <x:v>바클라바</x:v>
+      </x:c>
+      <x:c r="D48" s="23" t="str">
+        <x:v>Baklava</x:v>
+      </x:c>
+      <x:c r="E48" s="23" t="str">
+        <x:v>얇은 반죽층에 시럽과 견과류를 더한 이스탄불 대표 디저트로 소개된다.</x:v>
+      </x:c>
+      <x:c r="F48" s="23" t="str">
+        <x:v>미조사</x:v>
+      </x:c>
+      <x:c r="G48" s="23"/>
+      <x:c r="H48" s="23" t="str">
+        <x:v>대기</x:v>
+      </x:c>
+      <x:c r="I48" s="23" t="str">
+        <x:v>GoTürkiye</x:v>
+      </x:c>
+      <x:c r="J48" s="23" t="str">
+        <x:v>https://goturkiye.com/istanbul/the-sweet-happy-ever-after</x:v>
+      </x:c>
+      <x:c r="K48" s="23" t="str">
+        <x:v>관광청 음식 추천만 기록. 공식 판매 가격 표본은 별도로 확인하지 않아 가격대는 입력하지 않음.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="49" ht="44" customHeight="1">
+      <x:c r="A49" s="23" t="str">
+        <x:v>튀르키예</x:v>
+      </x:c>
+      <x:c r="B49" s="23" t="str">
+        <x:v>이스탄불</x:v>
+      </x:c>
+      <x:c r="C49" s="23" t="str">
+        <x:v>퀴네페</x:v>
+      </x:c>
+      <x:c r="D49" s="23" t="str">
+        <x:v>Künefe</x:v>
+      </x:c>
+      <x:c r="E49" s="23" t="str">
+        <x:v>따뜻하게 먹으며 안에 치즈를 넣는 튀르키예 디저트로 소개된다.</x:v>
+      </x:c>
+      <x:c r="F49" s="23" t="str">
+        <x:v>미조사</x:v>
+      </x:c>
+      <x:c r="G49" s="23"/>
+      <x:c r="H49" s="23" t="str">
+        <x:v>대기</x:v>
+      </x:c>
+      <x:c r="I49" s="23" t="str">
+        <x:v>GoTürkiye</x:v>
+      </x:c>
+      <x:c r="J49" s="23" t="str">
+        <x:v>https://goturkiye.com/istanbul/the-sweet-happy-ever-after</x:v>
+      </x:c>
+      <x:c r="K49" s="23" t="str">
+        <x:v>관광청 음식 추천만 기록. 공식 판매 가격 표본은 별도로 확인하지 않아 가격대는 입력하지 않음.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:K1"/>
@@ -15435,7 +17680,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rde74b1818f484788"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R932c66726412450c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -16507,7 +18752,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R133df445d96a4de7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra1a14d77eec2486a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>